<commit_message>
Update expert rubrics and revised test cases
</commit_message>
<xml_diff>
--- a/EL Agent测试集_260529_筛选后.xlsx
+++ b/EL Agent测试集_260529_筛选后.xlsx
@@ -3397,7 +3397,7 @@
       </c>
       <c r="F25" s="15" t="inlineStr">
         <is>
-          <t>我将上传一份报告，是关于GH组分变化验证的， 请你帮忙解读和分析，重点指出电压，效率和寿命的差异的原因。</t>
+          <t>请帮我总结下面这份报告的主要信息，要求逻辑框架清晰，关键数据充分。</t>
         </is>
       </c>
       <c r="G25" s="15" t="inlineStr">
@@ -3735,6 +3735,15 @@
 报告结论里写了 SGH5519，但表格主体是 SGH5516，我按 SGH5516 理解。
 REF 用的是 SFGD5501，目标体系用 SFGD5563，两者不能直接作为同一基准排序。
 最优绿光 EML 层组合推荐
+| 目标 | 	
+推荐 EML 组合 | PGD/FGD | 推荐比例 | 预期效率 | 预期 LT95@J25 | 是否满足目标 | 来源等级 / 置信度 | 主要依据与风险 |
+| 长寿命方案 | SGH5549:SGH5516 | SPGD508:SFGD5563=12%:0.7% | 5.7:4.3 | 约210–215 cd/A | 约90–100 h | 有机会满足，但窗口很窄 | B / 中 | 由 6:4 高寿命、低效率与 5:5 高效率、低寿命插值外推。6:4 实测 LT95&gt;100 h，但 CE&lt;210；5:5 CE&gt;220，但寿命不足。最佳折中点应靠近 5.6–5.8:4.4–4.2。风险是效率和寿命达标窗口极窄，需复验。 |
+| 高效率方案 | SGH5549:(SGH5516:N981) | SPGD508:SFGD5563=12%:0.7% | 4.8:(3.6:1.6)，即 P:N 总比约 4.8:5.2，N 内 SGH5516:N981≈7:3 | 目标240–245 cd/A | 目标70–80 h | 需实验验证 | C / 低-中 | 现有 4:6 效率最高但寿命只有25–33 h；说明 N-rich 有利效率但应力偏大。N981 的 T1=2.74 eV，高于 SGH5516 的2.58 eV，LUMO=-2.28 eV 也比 SGH5516 浅，有望降低激子/电子应力，同时保留部分 SGH5516 电子传输。风险是电压、复合区、能量转移效率需实测确认。 |
+我建议优先做 3 组 DOE：
+| 优先级EML | 方案 |目的 |
+| 1 | SGH5549:SGH5516=5.7:4.3 + SPGD508:SFGD5563=12%:0.7% | 冲击长寿命硬指标，验证 CE&gt;210、LT95&gt;90h 是否同时成立 |
+| 2 | SGH5549:SGH5516=5.6:4.4 + SPGD508:SFGD5563=12%:0.7% | 给长寿命方案留效率余量 |
+| 3 | SGH5549:(SGH5516:N981)=4.8:(7:3) + SPGD508:SFGD5563=12%:0.7% | 冲击高效率 &gt;240 cd/A，同时通过高 T1 N981 拉升寿命 |
 一句话建议：
 长寿命优先走 SGH5549:SGH5516≈5.7:4.3 微调；高效率目标仅靠现有 SGH5549:SGH5516 二元 P:N 很难达到，需要引入高 T1、浅 LUMO 的 N981 做三元 N-host 共混。</t>
         </is>

</xml_diff>